<commit_message>
Sube tabla de pines
</commit_message>
<xml_diff>
--- a/Controlador/Prototipo/pines.xlsx
+++ b/Controlador/Prototipo/pines.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="84">
   <si>
     <t>PC9</t>
   </si>
@@ -215,13 +215,64 @@
   </si>
   <si>
     <t>S. celdas</t>
+  </si>
+  <si>
+    <t>Banco</t>
+  </si>
+  <si>
+    <t>Señal</t>
+  </si>
+  <si>
+    <t>Pin MCU</t>
+  </si>
+  <si>
+    <t>Vc1</t>
+  </si>
+  <si>
+    <t>Banco 1</t>
+  </si>
+  <si>
+    <t>Vc2</t>
+  </si>
+  <si>
+    <t>Banco 2</t>
+  </si>
+  <si>
+    <t>Vc3</t>
+  </si>
+  <si>
+    <t>Celda</t>
+  </si>
+  <si>
+    <t>Vc_11</t>
+  </si>
+  <si>
+    <t>Vc_12</t>
+  </si>
+  <si>
+    <t>Vc_21</t>
+  </si>
+  <si>
+    <t>Vc_22</t>
+  </si>
+  <si>
+    <t>Vc_31</t>
+  </si>
+  <si>
+    <t>Vc_32</t>
+  </si>
+  <si>
+    <t>Banco 3</t>
+  </si>
+  <si>
+    <t>Pines morpho</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -231,6 +282,14 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -268,7 +327,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -276,17 +335,173 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -591,537 +806,709 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:K25"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B1">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E1">
-        <v>2</v>
-      </c>
-      <c r="H1">
-        <v>1</v>
-      </c>
-      <c r="I1" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1">
-        <v>2</v>
-      </c>
+    <row r="1" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D2" t="s">
-        <v>36</v>
+        <v>1</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="28" t="s">
+        <v>35</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>3</v>
-      </c>
-      <c r="I2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="J2" t="s">
-        <v>6</v>
+      <c r="I2" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>5</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D3" t="s">
-        <v>38</v>
+        <v>3</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>36</v>
       </c>
       <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="J3" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="H3">
-        <v>5</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="J3" t="s">
-        <v>7</v>
-      </c>
       <c r="K3">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4">
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <v>5</v>
+      </c>
+      <c r="I4" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="J4" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4">
-        <v>8</v>
-      </c>
-      <c r="H4">
-        <v>7</v>
-      </c>
-      <c r="I4" t="s">
-        <v>3</v>
-      </c>
-      <c r="J4" t="s">
-        <v>8</v>
-      </c>
       <c r="K4">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>40</v>
+        <v>7</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="30" t="s">
+        <v>4</v>
       </c>
       <c r="E5">
-        <v>10</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H5">
-        <v>9</v>
-      </c>
-      <c r="I5" t="s">
-        <v>4</v>
-      </c>
-      <c r="J5" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="I5" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>8</v>
       </c>
       <c r="K5">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6">
-        <v>11</v>
-      </c>
-      <c r="C6" t="s">
-        <v>41</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="30"/>
       <c r="E6">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>11</v>
-      </c>
-      <c r="J6" t="s">
-        <v>13</v>
+        <v>9</v>
+      </c>
+      <c r="I6" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="J6" s="17" t="s">
+        <v>9</v>
       </c>
       <c r="K6">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7">
+        <v>11</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="30"/>
+      <c r="E7">
+        <v>12</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>11</v>
+      </c>
+      <c r="I7" s="18"/>
+      <c r="J7" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E7">
-        <v>14</v>
-      </c>
-      <c r="F7">
-        <v>3</v>
-      </c>
-      <c r="H7">
-        <v>13</v>
-      </c>
-      <c r="J7" t="s">
-        <v>14</v>
-      </c>
       <c r="K7">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8">
-        <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D8" t="s">
-        <v>42</v>
+        <v>13</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="30" t="s">
+        <v>43</v>
       </c>
       <c r="E8">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H8">
-        <v>15</v>
-      </c>
-      <c r="J8" t="s">
-        <v>15</v>
+        <v>13</v>
+      </c>
+      <c r="I8" s="18"/>
+      <c r="J8" s="17" t="s">
+        <v>14</v>
       </c>
       <c r="K8">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>52</v>
+        <v>15</v>
+      </c>
+      <c r="C9" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>42</v>
       </c>
       <c r="E9">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H9">
-        <v>17</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="J9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="18"/>
+      <c r="J9" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="K9">
         <v>16</v>
-      </c>
-      <c r="K9">
-        <v>18</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10">
-        <v>19</v>
-      </c>
-      <c r="C10" t="s">
-        <v>4</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="30"/>
       <c r="E10">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H10">
-        <v>19</v>
-      </c>
-      <c r="I10" t="s">
-        <v>11</v>
-      </c>
-      <c r="J10" t="s">
         <v>17</v>
       </c>
+      <c r="I10" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="J10" s="19" t="s">
+        <v>16</v>
+      </c>
       <c r="K10">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11">
-        <v>21</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>53</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="C11" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="30"/>
       <c r="E11">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F11">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H11">
-        <v>21</v>
-      </c>
-      <c r="I11" t="s">
-        <v>12</v>
-      </c>
-      <c r="J11" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="I11" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="J11" s="17" t="s">
+        <v>17</v>
       </c>
       <c r="K11">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12">
-        <v>23</v>
-      </c>
-      <c r="C12" t="s">
-        <v>54</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="30"/>
       <c r="E12">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F12">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H12">
-        <v>23</v>
-      </c>
-      <c r="I12" t="s">
-        <v>23</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="I12" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="J12" s="17" t="s">
+        <v>18</v>
       </c>
       <c r="K12">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13">
-        <v>25</v>
-      </c>
-      <c r="C13" t="s">
-        <v>55</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="C13" s="29" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="30"/>
       <c r="E13">
-        <v>26</v>
+        <v>24</v>
+      </c>
+      <c r="F13">
+        <v>8</v>
       </c>
       <c r="H13">
-        <v>25</v>
-      </c>
-      <c r="I13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="K13">
         <v>24</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K13">
-        <v>26</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14">
-        <v>27</v>
-      </c>
-      <c r="C14" t="s">
-        <v>56</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>44</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="30"/>
       <c r="E14">
-        <v>28</v>
-      </c>
-      <c r="F14">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="H14">
-        <v>27</v>
-      </c>
-      <c r="I14" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J14" s="2" t="s">
-        <v>21</v>
+      <c r="I14" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="J14" s="21" t="s">
+        <v>20</v>
       </c>
       <c r="K14">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15">
-        <v>29</v>
-      </c>
-      <c r="C15" t="s">
-        <v>57</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>45</v>
+        <v>27</v>
+      </c>
+      <c r="C15" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="32" t="s">
+        <v>44</v>
       </c>
       <c r="E15">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>29</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>22</v>
+        <v>27</v>
+      </c>
+      <c r="I15" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="J15" s="21" t="s">
+        <v>21</v>
       </c>
       <c r="K15">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B16">
+        <v>29</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16">
+        <v>30</v>
+      </c>
+      <c r="F16">
+        <v>2</v>
+      </c>
+      <c r="H16">
+        <v>29</v>
+      </c>
+      <c r="I16" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="J16" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="K16">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B17">
         <v>31</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C17" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D17" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="E16">
+      <c r="E17">
         <v>32</v>
       </c>
-      <c r="F16">
+      <c r="F17">
         <v>3</v>
       </c>
-      <c r="H16">
+      <c r="H17">
         <v>31</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="I17" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="K16">
+      <c r="J17" s="17"/>
+      <c r="K17">
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B18">
         <v>33</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C18" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D18" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="E17">
+      <c r="E18">
         <v>34</v>
       </c>
-      <c r="F17">
+      <c r="F18">
         <v>4</v>
       </c>
-      <c r="H17">
+      <c r="H18">
         <v>33</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I18" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J18" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="K17">
+      <c r="K18">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B19">
         <v>35</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C19" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D19" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="E18">
+      <c r="E19">
         <v>36</v>
       </c>
-      <c r="F18">
+      <c r="F19">
         <v>5</v>
       </c>
-      <c r="H18">
+      <c r="H19">
         <v>35</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="I19" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J19" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="K18">
+      <c r="K19">
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B19">
+    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20">
         <v>37</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C20" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D20" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="E19">
+      <c r="E20">
         <v>38</v>
       </c>
-      <c r="F19">
+      <c r="F20">
         <v>6</v>
       </c>
-      <c r="H19">
+      <c r="H20">
         <v>37</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="I20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J20" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="K19">
+      <c r="K20">
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="C22" s="1"/>
-      <c r="D22" t="s">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C23" s="1"/>
+      <c r="D23" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="C23" s="2"/>
-      <c r="D23" t="s">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C24" s="2"/>
+      <c r="D24" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="C24" s="3"/>
-      <c r="D24" t="s">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C25" s="3"/>
+      <c r="D25" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="C25" s="5"/>
-      <c r="D25" t="s">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C26" s="4"/>
+      <c r="D26" t="s">
         <v>66</v>
       </c>
     </row>
+    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="8">
+        <v>1</v>
+      </c>
+      <c r="B35" s="9">
+        <v>1</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="8">
+        <v>1</v>
+      </c>
+      <c r="B36" s="9">
+        <v>2</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="8">
+        <v>2</v>
+      </c>
+      <c r="B37" s="9">
+        <v>1</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="8">
+        <v>2</v>
+      </c>
+      <c r="B38" s="9">
+        <v>2</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="8">
+        <v>3</v>
+      </c>
+      <c r="B39" s="9">
+        <v>1</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="11">
+        <v>3</v>
+      </c>
+      <c r="B40" s="12">
+        <v>2</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D40" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:K1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
probamos los leds, y ajustamos el controlador
</commit_message>
<xml_diff>
--- a/Controlador/Prototipo/pines.xlsx
+++ b/Controlador/Prototipo/pines.xlsx
@@ -419,7 +419,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -473,9 +473,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -495,11 +492,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -810,27 +813,27 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="D2" s="27" t="s">
         <v>35</v>
       </c>
       <c r="E2">
@@ -853,10 +856,10 @@
       <c r="B3">
         <v>3</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="30" t="s">
+      <c r="D3" s="29" t="s">
         <v>36</v>
       </c>
       <c r="E3">
@@ -879,10 +882,10 @@
       <c r="B4">
         <v>5</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="29" t="s">
         <v>38</v>
       </c>
       <c r="E4">
@@ -905,10 +908,10 @@
       <c r="B5">
         <v>7</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="29" t="s">
         <v>4</v>
       </c>
       <c r="E5">
@@ -931,10 +934,10 @@
       <c r="B6">
         <v>9</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="30"/>
+      <c r="D6" s="29"/>
       <c r="E6">
         <v>10</v>
       </c>
@@ -958,10 +961,10 @@
       <c r="B7">
         <v>11</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="30"/>
+      <c r="D7" s="29"/>
       <c r="E7">
         <v>12</v>
       </c>
@@ -971,7 +974,9 @@
       <c r="H7">
         <v>11</v>
       </c>
-      <c r="I7" s="18"/>
+      <c r="I7" s="35" t="s">
+        <v>20</v>
+      </c>
       <c r="J7" s="17" t="s">
         <v>13</v>
       </c>
@@ -983,10 +988,10 @@
       <c r="B8">
         <v>13</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D8" s="29" t="s">
         <v>43</v>
       </c>
       <c r="E8">
@@ -998,7 +1003,9 @@
       <c r="H8">
         <v>13</v>
       </c>
-      <c r="I8" s="18"/>
+      <c r="I8" s="35" t="s">
+        <v>21</v>
+      </c>
       <c r="J8" s="17" t="s">
         <v>14</v>
       </c>
@@ -1010,10 +1017,10 @@
       <c r="B9">
         <v>15</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="30" t="s">
+      <c r="D9" s="29" t="s">
         <v>42</v>
       </c>
       <c r="E9">
@@ -1025,8 +1032,10 @@
       <c r="H9">
         <v>15</v>
       </c>
-      <c r="I9" s="18"/>
-      <c r="J9" s="17" t="s">
+      <c r="I9" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="J9" s="19" t="s">
         <v>15</v>
       </c>
       <c r="K9">
@@ -1037,10 +1046,10 @@
       <c r="B10">
         <v>17</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="C10" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="30"/>
+      <c r="D10" s="29"/>
       <c r="E10">
         <v>18</v>
       </c>
@@ -1064,10 +1073,10 @@
       <c r="B11">
         <v>19</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="C11" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="D11" s="30"/>
+      <c r="D11" s="29"/>
       <c r="E11">
         <v>20</v>
       </c>
@@ -1091,10 +1100,10 @@
       <c r="B12">
         <v>21</v>
       </c>
-      <c r="C12" s="31" t="s">
+      <c r="C12" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="D12" s="30"/>
+      <c r="D12" s="29"/>
       <c r="E12">
         <v>22</v>
       </c>
@@ -1104,7 +1113,7 @@
       <c r="H12">
         <v>21</v>
       </c>
-      <c r="I12" s="18" t="s">
+      <c r="I12" s="35" t="s">
         <v>12</v>
       </c>
       <c r="J12" s="17" t="s">
@@ -1118,10 +1127,10 @@
       <c r="B13">
         <v>23</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="D13" s="30"/>
+      <c r="D13" s="29"/>
       <c r="E13">
         <v>24</v>
       </c>
@@ -1145,10 +1154,10 @@
       <c r="B14">
         <v>25</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="30"/>
+      <c r="D14" s="29"/>
       <c r="E14">
         <v>26</v>
       </c>
@@ -1158,9 +1167,7 @@
       <c r="I14" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="J14" s="21" t="s">
-        <v>20</v>
-      </c>
+      <c r="J14" s="29"/>
       <c r="K14">
         <v>26</v>
       </c>
@@ -1169,10 +1176,10 @@
       <c r="B15">
         <v>27</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="C15" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="30" t="s">
         <v>44</v>
       </c>
       <c r="E15">
@@ -1184,12 +1191,10 @@
       <c r="H15">
         <v>27</v>
       </c>
-      <c r="I15" s="22" t="s">
+      <c r="I15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="J15" s="21" t="s">
-        <v>21</v>
-      </c>
+      <c r="J15" s="29"/>
       <c r="K15">
         <v>28</v>
       </c>
@@ -1198,10 +1203,10 @@
       <c r="B16">
         <v>29</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="C16" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="D16" s="30" t="s">
         <v>45</v>
       </c>
       <c r="E16">
@@ -1213,12 +1218,10 @@
       <c r="H16">
         <v>29</v>
       </c>
-      <c r="I16" s="23" t="s">
+      <c r="I16" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="J16" s="20" t="s">
-        <v>22</v>
-      </c>
+      <c r="J16" s="29"/>
       <c r="K16">
         <v>30</v>
       </c>
@@ -1227,10 +1230,10 @@
       <c r="B17">
         <v>31</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C17" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="32" t="s">
+      <c r="D17" s="30" t="s">
         <v>46</v>
       </c>
       <c r="E17">
@@ -1242,7 +1245,7 @@
       <c r="H17">
         <v>31</v>
       </c>
-      <c r="I17" s="22" t="s">
+      <c r="I17" s="21" t="s">
         <v>26</v>
       </c>
       <c r="J17" s="17"/>
@@ -1254,10 +1257,10 @@
       <c r="B18">
         <v>33</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="D18" s="32" t="s">
+      <c r="D18" s="30" t="s">
         <v>47</v>
       </c>
       <c r="E18">
@@ -1269,7 +1272,7 @@
       <c r="H18">
         <v>33</v>
       </c>
-      <c r="I18" s="18" t="s">
+      <c r="I18" s="36" t="s">
         <v>27</v>
       </c>
       <c r="J18" s="17" t="s">
@@ -1283,10 +1286,10 @@
       <c r="B19">
         <v>35</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="C19" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="D19" s="32" t="s">
+      <c r="D19" s="30" t="s">
         <v>48</v>
       </c>
       <c r="E19">
@@ -1298,7 +1301,7 @@
       <c r="H19">
         <v>35</v>
       </c>
-      <c r="I19" s="24" t="s">
+      <c r="I19" s="23" t="s">
         <v>28</v>
       </c>
       <c r="J19" s="17" t="s">
@@ -1312,10 +1315,10 @@
       <c r="B20">
         <v>37</v>
       </c>
-      <c r="C20" s="33" t="s">
+      <c r="C20" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="D20" s="34" t="s">
+      <c r="D20" s="32" t="s">
         <v>49</v>
       </c>
       <c r="E20">
@@ -1327,10 +1330,10 @@
       <c r="H20">
         <v>37</v>
       </c>
-      <c r="I20" s="25" t="s">
+      <c r="I20" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="J20" s="26" t="s">
+      <c r="J20" s="25" t="s">
         <v>32</v>
       </c>
       <c r="K20">

</xml_diff>

<commit_message>
agrega funciones en controller, y cli
aun falta desarrollar mediciones y la logica del controlador. Ya estan la gran mayorias de las funciones preparadas en controlador solo queda unirlas
</commit_message>
<xml_diff>
--- a/Controlador/Prototipo/pines.xlsx
+++ b/Controlador/Prototipo/pines.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="99">
   <si>
     <t>PC9</t>
   </si>
@@ -266,6 +266,51 @@
   </si>
   <si>
     <t>Pines morpho</t>
+  </si>
+  <si>
+    <t>cell_21</t>
+  </si>
+  <si>
+    <t>bus_1</t>
+  </si>
+  <si>
+    <t>cell_11</t>
+  </si>
+  <si>
+    <t>cell_12</t>
+  </si>
+  <si>
+    <t>cell_22</t>
+  </si>
+  <si>
+    <t>PC0</t>
+  </si>
+  <si>
+    <t>cell_31</t>
+  </si>
+  <si>
+    <t>cell_32</t>
+  </si>
+  <si>
+    <t>PC1</t>
+  </si>
+  <si>
+    <t>out_neg</t>
+  </si>
+  <si>
+    <t>out_pos</t>
+  </si>
+  <si>
+    <t>bus_2</t>
+  </si>
+  <si>
+    <t>Pin ADC</t>
+  </si>
+  <si>
+    <t>Medición</t>
+  </si>
+  <si>
+    <t>A</t>
   </si>
 </sst>
 </file>
@@ -419,7 +464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -495,14 +540,36 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -809,22 +876,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="10" max="10" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
-      <c r="K1" s="33"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2">
@@ -974,7 +1044,7 @@
       <c r="H7">
         <v>11</v>
       </c>
-      <c r="I7" s="35" t="s">
+      <c r="I7" s="34" t="s">
         <v>20</v>
       </c>
       <c r="J7" s="17" t="s">
@@ -1003,7 +1073,7 @@
       <c r="H8">
         <v>13</v>
       </c>
-      <c r="I8" s="35" t="s">
+      <c r="I8" s="34" t="s">
         <v>21</v>
       </c>
       <c r="J8" s="17" t="s">
@@ -1032,7 +1102,7 @@
       <c r="H9">
         <v>15</v>
       </c>
-      <c r="I9" s="35" t="s">
+      <c r="I9" s="34" t="s">
         <v>22</v>
       </c>
       <c r="J9" s="19" t="s">
@@ -1100,7 +1170,7 @@
       <c r="B12">
         <v>21</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="33" t="s">
         <v>53</v>
       </c>
       <c r="D12" s="29"/>
@@ -1113,7 +1183,7 @@
       <c r="H12">
         <v>21</v>
       </c>
-      <c r="I12" s="35" t="s">
+      <c r="I12" s="34" t="s">
         <v>12</v>
       </c>
       <c r="J12" s="17" t="s">
@@ -1272,7 +1342,7 @@
       <c r="H18">
         <v>33</v>
       </c>
-      <c r="I18" s="36" t="s">
+      <c r="I18" s="35" t="s">
         <v>27</v>
       </c>
       <c r="J18" s="17" t="s">
@@ -1364,8 +1434,11 @@
         <v>66</v>
       </c>
     </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I27" s="36"/>
+    </row>
     <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>67</v>
       </c>
@@ -1375,6 +1448,7 @@
       <c r="C29" s="7" t="s">
         <v>69</v>
       </c>
+      <c r="F29" s="36"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
@@ -1386,6 +1460,12 @@
       <c r="C30" s="10" t="s">
         <v>26</v>
       </c>
+      <c r="F30" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="G30" s="43" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
@@ -1397,6 +1477,12 @@
       <c r="C31" s="10" t="s">
         <v>25</v>
       </c>
+      <c r="F31" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="G31" s="40" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
@@ -1408,9 +1494,22 @@
       <c r="C32" s="13" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F32" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="G32" s="40" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F33" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="G33" s="40" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>67</v>
       </c>
@@ -1423,8 +1522,14 @@
       <c r="D34" s="7" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F34" s="38" t="s">
+        <v>47</v>
+      </c>
+      <c r="G34" s="40" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="8">
         <v>1</v>
       </c>
@@ -1437,8 +1542,17 @@
       <c r="D35" s="10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F35" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="G35" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="I35" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="8">
         <v>1</v>
       </c>
@@ -1451,8 +1565,14 @@
       <c r="D36" s="10" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F36" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="G36" s="40" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="8">
         <v>2</v>
       </c>
@@ -1465,8 +1585,14 @@
       <c r="D37" s="10" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F37" s="38" t="s">
+        <v>20</v>
+      </c>
+      <c r="G37" s="40" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
         <v>2</v>
       </c>
@@ -1479,8 +1605,14 @@
       <c r="D38" s="10" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F38" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G38" s="40" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="8">
         <v>3</v>
       </c>
@@ -1493,8 +1625,14 @@
       <c r="D39" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F39" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="G39" s="40" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="11">
         <v>3</v>
       </c>
@@ -1507,6 +1645,19 @@
       <c r="D40" s="13" t="s">
         <v>16</v>
       </c>
+      <c r="F40" s="39" t="s">
+        <v>30</v>
+      </c>
+      <c r="G40" s="41" t="s">
+        <v>95</v>
+      </c>
+      <c r="I40" s="37"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I41" s="36"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I42" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
inicializa todos los pines del gpio en low
</commit_message>
<xml_diff>
--- a/Controlador/Prototipo/pines.xlsx
+++ b/Controlador/Prototipo/pines.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView minimized="1" xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="98">
   <si>
     <t>PC9</t>
   </si>
@@ -308,9 +308,6 @@
   </si>
   <si>
     <t>Medición</t>
-  </si>
-  <si>
-    <t>A</t>
   </si>
 </sst>
 </file>
@@ -1548,9 +1545,6 @@
       <c r="G35" s="40" t="s">
         <v>90</v>
       </c>
-      <c r="I35" t="s">
-        <v>98</v>
-      </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="8">

</xml_diff>